<commit_message>
stabalized the Dataset creation by waiting for notification to get it success
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052/UK_ImportCoA.xlsx
+++ b/Test Data/Regression/4689052/UK_ImportCoA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ATHENA_Automation_1.0\Workbook_Automation\src\OCT\TestData\SmokeBVT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Playwright_self\playwright-OCT-Automation2\Test Data\Regression\4689052\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2429E39B-3CF1-45AB-AA85-80B8B9B7117A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52030C86-DF21-43AF-80C7-DEEB87B1D182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{DA4B9D26-82E2-4448-9864-B6C60423C710}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DA4B9D26-82E2-4448-9864-B6C60423C710}"/>
   </bookViews>
   <sheets>
     <sheet name="Trial balance" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
   <si>
     <t>Corporation tax charge</t>
   </si>
@@ -98,9 +98,6 @@
     <t>Staff training</t>
   </si>
   <si>
-    <t>Printing, postage and stationery</t>
-  </si>
-  <si>
     <t>Computer software and maintenance costs</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
   </si>
   <si>
     <t>Rent</t>
-  </si>
-  <si>
-    <t>Rent and rates</t>
   </si>
   <si>
     <t>Redundancy costs</t>
@@ -239,9 +233,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,7 +273,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -385,7 +379,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -527,7 +521,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -535,7 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70E64DCE-4436-4400-B4EF-16C303003D7A}">
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="56.1796875" bestFit="1" customWidth="1"/>
@@ -543,10 +537,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -554,7 +548,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -562,7 +556,7 @@
         <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -570,7 +564,7 @@
         <v>60</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -578,7 +572,7 @@
         <v>70</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -586,7 +580,7 @@
         <v>71</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -594,7 +588,7 @@
         <v>74</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -602,7 +596,7 @@
         <v>77</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -610,7 +604,7 @@
         <v>230</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -618,7 +612,7 @@
         <v>231</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -626,7 +620,7 @@
         <v>232</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -634,7 +628,7 @@
         <v>234</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -642,7 +636,7 @@
         <v>243</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -650,7 +644,7 @@
         <v>244</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -658,238 +652,222 @@
         <v>248</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
-        <v>301</v>
+        <v>330</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
-        <v>310</v>
+        <v>335</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
-        <v>365</v>
+        <v>374</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
-        <v>370</v>
+        <v>386</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
-        <v>374</v>
+        <v>405</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
-        <v>386</v>
+        <v>431</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
-        <v>405</v>
+        <v>444</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
-        <v>431</v>
+        <v>470</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" s="2">
-        <v>444</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" s="2">
-        <v>470</v>
-      </c>
-      <c r="B44" s="2" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>